<commit_message>
Fix static templates: add date+narration to opening stock, add sales invoice template
- templates/template-3-opening-stock.xlsx now header item_name,qty,rate,date,narration (was missing date)
- templates/template-5-sales-invoices.xlsx new with invoice_no,date,buyer_name,buyer_gstin,item_name,qty,rate,gst_rate etc for PI-200 import
- ensures both dynamic /api/export and static templates match

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/templates/template-3-opening-stock.xlsx
+++ b/templates/template-3-opening-stock.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:E2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,28 +410,40 @@
       <c r="C1" t="str">
         <v>rate</v>
       </c>
+      <c r="D1" t="str">
+        <v>date</v>
+      </c>
+      <c r="E1" t="str">
+        <v>narration</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>EXAMPLE — delete this row</v>
       </c>
-      <c r="B2" t="str">
-        <v/>
-      </c>
-      <c r="C2" t="str">
-        <v/>
+      <c r="B2">
+        <v>100</v>
+      </c>
+      <c r="C2">
+        <v>80.5</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2026-09-10</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Batch A / Supplier XYZ</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A3"/>
   <cols>
     <col min="1" max="1" width="110.83203125" customWidth="1"/>
   </cols>
@@ -441,9 +453,19 @@
         <v>Fill one item per row. Required: item_name (must exist), qty, rate.</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Optional: date = date of buying YYYY-MM-DD for tracking buy vs sell age. If blank, uses the date you choose in the import screen.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Optional: narration = batch / supplier ref.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>